<commit_message>
datos: 2026-05 (mayo) - AIF/IMIG consolidados + IPC actualizado
</commit_message>
<xml_diff>
--- a/data/reference/IPC.xlsx
+++ b/data/reference/IPC.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sriverti\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sriverti\Desktop\INECO\Repositorios\cuentas_publicas\data\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D26A2E2-D630-4A1B-B5C2-1E23A046A739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A90F7D-B790-445D-A271-2FDCAC7EDD34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -429,7 +429,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:P986"/>
+  <dimension ref="A1:P985"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.28515625" customWidth="1"/>
@@ -5530,7 +5530,50 @@
       <c r="O113" s="9"/>
       <c r="P113" s="13"/>
     </row>
-    <row r="114" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="114" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="10">
+        <v>46143</v>
+      </c>
+      <c r="B114" s="12">
+        <v>11607.393700000001</v>
+      </c>
+      <c r="C114" s="12">
+        <v>12494.976699999999</v>
+      </c>
+      <c r="D114" s="12">
+        <v>8033.2555000000002</v>
+      </c>
+      <c r="E114" s="12">
+        <v>8350.2423999999992</v>
+      </c>
+      <c r="F114" s="12">
+        <v>12790.077600000001</v>
+      </c>
+      <c r="G114" s="12">
+        <v>9312.2108000000007</v>
+      </c>
+      <c r="H114" s="12">
+        <v>12832.0291</v>
+      </c>
+      <c r="I114" s="12">
+        <v>12330.501700000001</v>
+      </c>
+      <c r="J114" s="12">
+        <v>10838.4277</v>
+      </c>
+      <c r="K114" s="12">
+        <v>10132.370500000001</v>
+      </c>
+      <c r="L114" s="12">
+        <v>10840.9295</v>
+      </c>
+      <c r="M114" s="12">
+        <v>14291.4848</v>
+      </c>
+      <c r="N114" s="12">
+        <v>11171.6219</v>
+      </c>
+    </row>
     <row r="115" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="116" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="117" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -6402,7 +6445,6 @@
     <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>